<commit_message>
Add Map View, Percentage Calculator, Ecclesiastical, News Search, Teams mirrors; extend Dynamics 365 mirror; rebuild Pass Back Form layout
</commit_message>
<xml_diff>
--- a/fixtures/Pass Back Form.xlsx
+++ b/fixtures/Pass Back Form.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:E229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -428,93 +428,158 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="3">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Underwriter</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Automated Renewal Review</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="D3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Underwriting Authority Level</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Referral Required</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="C44" t="inlineStr">
         <is>
           <t>Claims Prior to Reception</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="D44" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Intruder Alarm Details</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Police Response</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Rationale</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Referral Required</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="B190" t="inlineStr">
         <is>
           <t>Has the Insured Opted Pool Re?</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="C190" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="B194" t="inlineStr">
         <is>
           <t>Flood/FloodRe Rationale</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="C194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Referral Required</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="C197" t="inlineStr">
         <is>
           <t>Reinsurance</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Rationale</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>This renewal is being passed back for manual review due to the presence of Subject to Survey Clause H0054 and because Renewal method (02) requires manual evaluation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
+      <c r="D197" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Referral Required</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Referral Required</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Standard Commission Paid</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Excess</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Book Premium</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Book Premium Minus ENBP</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Risk Profile</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>